<commit_message>
Updated vehicle weight estimates to include updated parts post crash
</commit_message>
<xml_diff>
--- a/CAD/Test Stand V2.1/vehicle_weight V2.xlsx
+++ b/CAD/Test Stand V2.1/vehicle_weight V2.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Projects\Propulsive Lander\CAD\Test Stand V2.1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LoneHunter13\OneDrive\Documents\Projects\Propulsive Lander\CAD\Test Stand V2.1\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="12945" windowHeight="8430"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="12950" windowHeight="8430"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="70">
   <si>
     <t>Test Frame</t>
   </si>
@@ -222,6 +222,18 @@
   </si>
   <si>
     <t>Needs Updating</t>
+  </si>
+  <si>
+    <t>Version 2.1 Estimate (Hover Testing Config, POST CRASH UPDATES)</t>
+  </si>
+  <si>
+    <t>Bottom Deck (Updated)</t>
+  </si>
+  <si>
+    <t>Upper Deck (Updated)</t>
+  </si>
+  <si>
+    <t>Gimbal Ring (Updated)</t>
   </si>
 </sst>
 </file>
@@ -566,23 +578,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L117"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:L137"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="3.7109375" style="2" customWidth="1"/>
-    <col min="7" max="7" width="27.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="3.7265625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="27.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.26953125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="18" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -597,7 +609,7 @@
       <c r="J1" s="5"/>
       <c r="K1" s="5"/>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -623,7 +635,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -649,7 +661,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -675,7 +687,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -702,7 +714,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -728,7 +740,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -754,7 +766,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
@@ -780,7 +792,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>23</v>
       </c>
@@ -806,7 +818,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>22</v>
       </c>
@@ -832,7 +844,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="D11" t="s">
         <v>20</v>
       </c>
@@ -846,7 +858,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -874,7 +886,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="D13" t="s">
         <v>4</v>
       </c>
@@ -888,7 +900,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="D14" t="s">
         <v>21</v>
       </c>
@@ -902,7 +914,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="D15" t="s">
         <v>15</v>
       </c>
@@ -910,7 +922,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="D16" t="s">
         <v>7</v>
       </c>
@@ -918,7 +930,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="4:11" x14ac:dyDescent="0.35">
       <c r="D17" t="s">
         <v>8</v>
       </c>
@@ -933,7 +945,7 @@
         <v>587</v>
       </c>
     </row>
-    <row r="18" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="4:11" x14ac:dyDescent="0.35">
       <c r="D18" t="s">
         <v>27</v>
       </c>
@@ -941,7 +953,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="4:11" x14ac:dyDescent="0.35">
       <c r="D19" t="s">
         <v>14</v>
       </c>
@@ -956,7 +968,7 @@
         <v>938</v>
       </c>
     </row>
-    <row r="20" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="4:11" x14ac:dyDescent="0.35">
       <c r="D20" t="s">
         <v>16</v>
       </c>
@@ -964,7 +976,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="21" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="4:11" x14ac:dyDescent="0.35">
       <c r="D21" t="s">
         <v>6</v>
       </c>
@@ -979,7 +991,7 @@
       <c r="J21" s="5"/>
       <c r="K21" s="5"/>
     </row>
-    <row r="22" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="4:11" x14ac:dyDescent="0.35">
       <c r="G22" t="s">
         <v>28</v>
       </c>
@@ -993,7 +1005,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="4:11" x14ac:dyDescent="0.35">
       <c r="D23" t="s">
         <v>17</v>
       </c>
@@ -1013,7 +1025,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="24" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="4:11" x14ac:dyDescent="0.35">
       <c r="D24" t="s">
         <v>6</v>
       </c>
@@ -1033,7 +1045,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="4:11" x14ac:dyDescent="0.35">
       <c r="D25" t="s">
         <v>26</v>
       </c>
@@ -1053,7 +1065,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="26" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="4:11" x14ac:dyDescent="0.35">
       <c r="D26" t="s">
         <v>25</v>
       </c>
@@ -1073,7 +1085,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="4:11" x14ac:dyDescent="0.35">
       <c r="G27" s="3" t="s">
         <v>7</v>
       </c>
@@ -1087,7 +1099,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="28" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="4:11" x14ac:dyDescent="0.35">
       <c r="D28" t="s">
         <v>9</v>
       </c>
@@ -1108,7 +1120,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="29" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="4:11" x14ac:dyDescent="0.35">
       <c r="G29" t="s">
         <v>6</v>
       </c>
@@ -1122,7 +1134,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="30" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="4:11" x14ac:dyDescent="0.35">
       <c r="D30" t="s">
         <v>33</v>
       </c>
@@ -1140,7 +1152,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="31" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="4:11" x14ac:dyDescent="0.35">
       <c r="J31" t="s">
         <v>27</v>
       </c>
@@ -1148,7 +1160,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="32" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="4:11" x14ac:dyDescent="0.35">
       <c r="G32" t="s">
         <v>9</v>
       </c>
@@ -1163,7 +1175,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="33" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="4:11" x14ac:dyDescent="0.35">
       <c r="D33" t="s">
         <v>35</v>
       </c>
@@ -1177,7 +1189,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="34" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="4:11" x14ac:dyDescent="0.35">
       <c r="D34" t="s">
         <v>36</v>
       </c>
@@ -1191,7 +1203,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="35" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="4:11" x14ac:dyDescent="0.35">
       <c r="J35" t="s">
         <v>32</v>
       </c>
@@ -1200,7 +1212,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="36" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="4:11" x14ac:dyDescent="0.35">
       <c r="D36" t="s">
         <v>37</v>
       </c>
@@ -1215,7 +1227,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="38" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="4:11" x14ac:dyDescent="0.35">
       <c r="J38" t="s">
         <v>9</v>
       </c>
@@ -1224,7 +1236,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="39" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="4:11" x14ac:dyDescent="0.35">
       <c r="G39" t="s">
         <v>30</v>
       </c>
@@ -1233,7 +1245,7 @@
         <v>862</v>
       </c>
     </row>
-    <row r="41" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="4:11" x14ac:dyDescent="0.35">
       <c r="G41" s="5" t="s">
         <v>59</v>
       </c>
@@ -1242,7 +1254,7 @@
       <c r="J41" s="5"/>
       <c r="K41" s="5"/>
     </row>
-    <row r="42" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="4:11" x14ac:dyDescent="0.35">
       <c r="G42" t="s">
         <v>28</v>
       </c>
@@ -1256,7 +1268,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="4:11" x14ac:dyDescent="0.35">
       <c r="G43" t="s">
         <v>39</v>
       </c>
@@ -1271,7 +1283,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="44" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="4:11" x14ac:dyDescent="0.35">
       <c r="G44" t="s">
         <v>40</v>
       </c>
@@ -1285,7 +1297,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="45" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="4:11" x14ac:dyDescent="0.35">
       <c r="G45" t="s">
         <v>41</v>
       </c>
@@ -1299,7 +1311,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="46" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="46" spans="4:11" x14ac:dyDescent="0.35">
       <c r="G46" t="s">
         <v>43</v>
       </c>
@@ -1315,7 +1327,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="47" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="4:11" x14ac:dyDescent="0.35">
       <c r="G47" t="s">
         <v>42</v>
       </c>
@@ -1331,7 +1343,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="48" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="48" spans="4:11" x14ac:dyDescent="0.35">
       <c r="G48" t="s">
         <v>44</v>
       </c>
@@ -1346,7 +1358,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="49" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="49" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G49" t="s">
         <v>45</v>
       </c>
@@ -1360,7 +1372,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="50" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="50" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G50" t="s">
         <v>47</v>
       </c>
@@ -1375,7 +1387,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="51" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="51" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G51" t="s">
         <v>53</v>
       </c>
@@ -1389,7 +1401,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="52" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="52" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G52" t="s">
         <v>54</v>
       </c>
@@ -1403,7 +1415,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="53" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="53" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G53" t="s">
         <v>55</v>
       </c>
@@ -1417,7 +1429,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="54" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="54" spans="7:11" x14ac:dyDescent="0.35">
       <c r="J54" t="s">
         <v>20</v>
       </c>
@@ -1426,7 +1438,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="55" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="55" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G55" t="s">
         <v>9</v>
       </c>
@@ -1435,7 +1447,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="56" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="56" spans="7:11" x14ac:dyDescent="0.35">
       <c r="J56" t="s">
         <v>9</v>
       </c>
@@ -1444,7 +1456,7 @@
         <v>645</v>
       </c>
     </row>
-    <row r="58" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="58" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G58" t="s">
         <v>56</v>
       </c>
@@ -1453,7 +1465,7 @@
         <v>861</v>
       </c>
     </row>
-    <row r="61" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="61" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G61" s="5" t="s">
         <v>60</v>
       </c>
@@ -1462,7 +1474,7 @@
       <c r="J61" s="5"/>
       <c r="K61" s="5"/>
     </row>
-    <row r="62" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="62" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G62" t="s">
         <v>28</v>
       </c>
@@ -1476,7 +1488,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="63" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="63" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G63" t="s">
         <v>39</v>
       </c>
@@ -1491,7 +1503,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="64" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="64" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G64" t="s">
         <v>40</v>
       </c>
@@ -1505,7 +1517,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="65" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="65" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G65" t="s">
         <v>41</v>
       </c>
@@ -1519,7 +1531,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="66" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="66" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G66" t="s">
         <v>43</v>
       </c>
@@ -1535,7 +1547,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="67" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="67" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G67" t="s">
         <v>42</v>
       </c>
@@ -1551,7 +1563,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="68" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="68" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G68" t="s">
         <v>44</v>
       </c>
@@ -1566,7 +1578,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="69" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="69" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G69" t="s">
         <v>45</v>
       </c>
@@ -1580,7 +1592,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="70" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="70" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G70" t="s">
         <v>47</v>
       </c>
@@ -1595,7 +1607,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="71" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="71" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G71" s="3" t="s">
         <v>53</v>
       </c>
@@ -1609,7 +1621,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="72" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="72" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G72" s="3" t="s">
         <v>54</v>
       </c>
@@ -1623,7 +1635,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="73" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="73" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G73" t="s">
         <v>55</v>
       </c>
@@ -1637,7 +1649,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="74" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="74" spans="7:11" x14ac:dyDescent="0.35">
       <c r="J74" t="s">
         <v>20</v>
       </c>
@@ -1646,7 +1658,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="75" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="75" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G75" t="s">
         <v>9</v>
       </c>
@@ -1655,7 +1667,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="76" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="76" spans="7:11" x14ac:dyDescent="0.35">
       <c r="J76" t="s">
         <v>9</v>
       </c>
@@ -1664,7 +1676,7 @@
         <v>645</v>
       </c>
     </row>
-    <row r="78" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="78" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G78" t="s">
         <v>56</v>
       </c>
@@ -1673,7 +1685,7 @@
         <v>829</v>
       </c>
     </row>
-    <row r="80" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="80" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G80" s="5" t="s">
         <v>57</v>
       </c>
@@ -1682,7 +1694,7 @@
       <c r="J80" s="5"/>
       <c r="K80" s="5"/>
     </row>
-    <row r="81" spans="7:12" x14ac:dyDescent="0.25">
+    <row r="81" spans="7:12" x14ac:dyDescent="0.35">
       <c r="G81" t="s">
         <v>28</v>
       </c>
@@ -1696,7 +1708,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="82" spans="7:12" x14ac:dyDescent="0.25">
+    <row r="82" spans="7:12" x14ac:dyDescent="0.35">
       <c r="G82" t="s">
         <v>39</v>
       </c>
@@ -1711,7 +1723,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="83" spans="7:12" x14ac:dyDescent="0.25">
+    <row r="83" spans="7:12" x14ac:dyDescent="0.35">
       <c r="G83" t="s">
         <v>40</v>
       </c>
@@ -1725,7 +1737,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="84" spans="7:12" x14ac:dyDescent="0.25">
+    <row r="84" spans="7:12" x14ac:dyDescent="0.35">
       <c r="G84" t="s">
         <v>41</v>
       </c>
@@ -1739,7 +1751,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="85" spans="7:12" x14ac:dyDescent="0.25">
+    <row r="85" spans="7:12" x14ac:dyDescent="0.35">
       <c r="G85" t="s">
         <v>43</v>
       </c>
@@ -1755,7 +1767,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="86" spans="7:12" x14ac:dyDescent="0.25">
+    <row r="86" spans="7:12" x14ac:dyDescent="0.35">
       <c r="G86" t="s">
         <v>61</v>
       </c>
@@ -1770,7 +1782,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="87" spans="7:12" x14ac:dyDescent="0.25">
+    <row r="87" spans="7:12" x14ac:dyDescent="0.35">
       <c r="G87" t="s">
         <v>44</v>
       </c>
@@ -1785,7 +1797,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="88" spans="7:12" x14ac:dyDescent="0.25">
+    <row r="88" spans="7:12" x14ac:dyDescent="0.35">
       <c r="G88" t="s">
         <v>45</v>
       </c>
@@ -1799,7 +1811,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="89" spans="7:12" x14ac:dyDescent="0.25">
+    <row r="89" spans="7:12" x14ac:dyDescent="0.35">
       <c r="G89" t="s">
         <v>47</v>
       </c>
@@ -1814,7 +1826,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="90" spans="7:12" x14ac:dyDescent="0.25">
+    <row r="90" spans="7:12" x14ac:dyDescent="0.35">
       <c r="G90" t="s">
         <v>53</v>
       </c>
@@ -1828,7 +1840,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="7:12" x14ac:dyDescent="0.25">
+    <row r="91" spans="7:12" x14ac:dyDescent="0.35">
       <c r="G91" t="s">
         <v>54</v>
       </c>
@@ -1842,7 +1854,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="92" spans="7:12" x14ac:dyDescent="0.25">
+    <row r="92" spans="7:12" x14ac:dyDescent="0.35">
       <c r="G92" s="4" t="s">
         <v>55</v>
       </c>
@@ -1859,7 +1871,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="93" spans="7:12" x14ac:dyDescent="0.25">
+    <row r="93" spans="7:12" x14ac:dyDescent="0.35">
       <c r="J93" t="s">
         <v>63</v>
       </c>
@@ -1867,7 +1879,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="94" spans="7:12" x14ac:dyDescent="0.25">
+    <row r="94" spans="7:12" x14ac:dyDescent="0.35">
       <c r="G94" t="s">
         <v>9</v>
       </c>
@@ -1882,7 +1894,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="95" spans="7:12" x14ac:dyDescent="0.25">
+    <row r="95" spans="7:12" x14ac:dyDescent="0.35">
       <c r="J95" s="4" t="s">
         <v>20</v>
       </c>
@@ -1894,7 +1906,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="96" spans="7:12" x14ac:dyDescent="0.25">
+    <row r="96" spans="7:12" x14ac:dyDescent="0.35">
       <c r="J96" t="s">
         <v>9</v>
       </c>
@@ -1903,7 +1915,7 @@
         <v>742</v>
       </c>
     </row>
-    <row r="97" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="97" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G97" t="s">
         <v>56</v>
       </c>
@@ -1912,7 +1924,7 @@
         <v>975</v>
       </c>
     </row>
-    <row r="100" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="100" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G100" s="5" t="s">
         <v>58</v>
       </c>
@@ -1921,7 +1933,7 @@
       <c r="J100" s="5"/>
       <c r="K100" s="5"/>
     </row>
-    <row r="101" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="101" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G101" t="s">
         <v>28</v>
       </c>
@@ -1935,7 +1947,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="102" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="102" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G102" t="s">
         <v>39</v>
       </c>
@@ -1950,7 +1962,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="103" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="103" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G103" t="s">
         <v>40</v>
       </c>
@@ -1964,7 +1976,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="104" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="104" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G104" t="s">
         <v>41</v>
       </c>
@@ -1978,7 +1990,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="105" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="105" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G105" t="s">
         <v>43</v>
       </c>
@@ -1994,7 +2006,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="106" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="106" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G106" t="s">
         <v>42</v>
       </c>
@@ -2009,7 +2021,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="107" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="107" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G107" t="s">
         <v>44</v>
       </c>
@@ -2024,7 +2036,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="108" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="108" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G108" t="s">
         <v>45</v>
       </c>
@@ -2038,7 +2050,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="109" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="109" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G109" t="s">
         <v>47</v>
       </c>
@@ -2053,7 +2065,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="110" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="110" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G110" s="3" t="s">
         <v>53</v>
       </c>
@@ -2067,7 +2079,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="111" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G111" s="3" t="s">
         <v>54</v>
       </c>
@@ -2081,7 +2093,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="112" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="112" spans="7:11" x14ac:dyDescent="0.35">
       <c r="G112" s="4" t="s">
         <v>55</v>
       </c>
@@ -2098,7 +2110,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="113" spans="7:12" x14ac:dyDescent="0.25">
+    <row r="113" spans="7:12" x14ac:dyDescent="0.35">
       <c r="J113" t="s">
         <v>63</v>
       </c>
@@ -2106,7 +2118,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="114" spans="7:12" x14ac:dyDescent="0.25">
+    <row r="114" spans="7:12" x14ac:dyDescent="0.35">
       <c r="G114" t="s">
         <v>9</v>
       </c>
@@ -2121,7 +2133,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="115" spans="7:12" x14ac:dyDescent="0.25">
+    <row r="115" spans="7:12" x14ac:dyDescent="0.35">
       <c r="J115" s="4" t="s">
         <v>20</v>
       </c>
@@ -2133,7 +2145,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="116" spans="7:12" x14ac:dyDescent="0.25">
+    <row r="116" spans="7:12" x14ac:dyDescent="0.35">
       <c r="J116" t="s">
         <v>9</v>
       </c>
@@ -2142,7 +2154,7 @@
         <v>740</v>
       </c>
     </row>
-    <row r="117" spans="7:12" x14ac:dyDescent="0.25">
+    <row r="117" spans="7:12" x14ac:dyDescent="0.35">
       <c r="G117" t="s">
         <v>56</v>
       </c>
@@ -2151,8 +2163,249 @@
         <v>941</v>
       </c>
     </row>
+    <row r="120" spans="7:12" x14ac:dyDescent="0.35">
+      <c r="G120" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="H120" s="5"/>
+      <c r="I120" s="5"/>
+      <c r="J120" s="5"/>
+      <c r="K120" s="5"/>
+    </row>
+    <row r="121" spans="7:12" x14ac:dyDescent="0.35">
+      <c r="G121" t="s">
+        <v>28</v>
+      </c>
+      <c r="H121" t="s">
+        <v>3</v>
+      </c>
+      <c r="J121" t="s">
+        <v>29</v>
+      </c>
+      <c r="K121" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="122" spans="7:12" x14ac:dyDescent="0.35">
+      <c r="G122" t="s">
+        <v>39</v>
+      </c>
+      <c r="H122">
+        <v>8</v>
+      </c>
+      <c r="J122" t="s">
+        <v>46</v>
+      </c>
+      <c r="K122">
+        <f>45*2</f>
+        <v>90</v>
+      </c>
+    </row>
+    <row r="123" spans="7:12" x14ac:dyDescent="0.35">
+      <c r="G123" t="s">
+        <v>67</v>
+      </c>
+      <c r="H123">
+        <v>42</v>
+      </c>
+      <c r="J123" t="s">
+        <v>11</v>
+      </c>
+      <c r="K123">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="124" spans="7:12" x14ac:dyDescent="0.35">
+      <c r="G124" t="s">
+        <v>68</v>
+      </c>
+      <c r="H124">
+        <f>133-K129-K131-K132-K127-1</f>
+        <v>53</v>
+      </c>
+      <c r="J124" t="s">
+        <v>48</v>
+      </c>
+      <c r="K124">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="125" spans="7:12" x14ac:dyDescent="0.35">
+      <c r="G125" t="s">
+        <v>43</v>
+      </c>
+      <c r="H125">
+        <f>2*17</f>
+        <v>34</v>
+      </c>
+      <c r="J125" t="s">
+        <v>49</v>
+      </c>
+      <c r="K125">
+        <f>2*48</f>
+        <v>96</v>
+      </c>
+    </row>
+    <row r="126" spans="7:12" x14ac:dyDescent="0.35">
+      <c r="G126" t="s">
+        <v>61</v>
+      </c>
+      <c r="H126">
+        <f>4*5</f>
+        <v>20</v>
+      </c>
+      <c r="J126" t="s">
+        <v>16</v>
+      </c>
+      <c r="K126">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="127" spans="7:12" x14ac:dyDescent="0.35">
+      <c r="G127" t="s">
+        <v>44</v>
+      </c>
+      <c r="H127">
+        <f>2*15</f>
+        <v>30</v>
+      </c>
+      <c r="J127" t="s">
+        <v>18</v>
+      </c>
+      <c r="K127">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="128" spans="7:12" x14ac:dyDescent="0.35">
+      <c r="G128" t="s">
+        <v>69</v>
+      </c>
+      <c r="H128">
+        <v>4</v>
+      </c>
+      <c r="J128" t="s">
+        <v>19</v>
+      </c>
+      <c r="K128">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="129" spans="7:12" x14ac:dyDescent="0.35">
+      <c r="G129" t="s">
+        <v>47</v>
+      </c>
+      <c r="H129">
+        <v>1</v>
+      </c>
+      <c r="J129" t="s">
+        <v>21</v>
+      </c>
+      <c r="K129">
+        <f>76/2</f>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="130" spans="7:12" x14ac:dyDescent="0.35">
+      <c r="G130" t="s">
+        <v>53</v>
+      </c>
+      <c r="H130">
+        <v>12</v>
+      </c>
+      <c r="J130" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="K130">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131" spans="7:12" x14ac:dyDescent="0.35">
+      <c r="G131" t="s">
+        <v>54</v>
+      </c>
+      <c r="H131">
+        <v>16</v>
+      </c>
+      <c r="J131" t="s">
+        <v>51</v>
+      </c>
+      <c r="K131">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="132" spans="7:12" x14ac:dyDescent="0.35">
+      <c r="G132" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="H132" s="4">
+        <v>42</v>
+      </c>
+      <c r="I132" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="J132" t="s">
+        <v>62</v>
+      </c>
+      <c r="K132">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="133" spans="7:12" x14ac:dyDescent="0.35">
+      <c r="J133" t="s">
+        <v>63</v>
+      </c>
+      <c r="K133">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="134" spans="7:12" x14ac:dyDescent="0.35">
+      <c r="G134" t="s">
+        <v>9</v>
+      </c>
+      <c r="H134">
+        <f>SUM(H122:H132)</f>
+        <v>262</v>
+      </c>
+      <c r="J134" t="s">
+        <v>64</v>
+      </c>
+      <c r="K134">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="135" spans="7:12" x14ac:dyDescent="0.35">
+      <c r="J135" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K135" s="4">
+        <f>(2/4)*22</f>
+        <v>11</v>
+      </c>
+      <c r="L135" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="136" spans="7:12" x14ac:dyDescent="0.35">
+      <c r="J136" t="s">
+        <v>9</v>
+      </c>
+      <c r="K136">
+        <f>SUM(K122:K135)</f>
+        <v>742</v>
+      </c>
+    </row>
+    <row r="137" spans="7:12" x14ac:dyDescent="0.35">
+      <c r="G137" t="s">
+        <v>56</v>
+      </c>
+      <c r="H137">
+        <f>SUM(H134,K136)</f>
+        <v>1004</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
+    <mergeCell ref="G120:K120"/>
     <mergeCell ref="G100:K100"/>
     <mergeCell ref="G61:K61"/>
     <mergeCell ref="G1:K1"/>

</xml_diff>